<commit_message>
removal of extra dates
</commit_message>
<xml_diff>
--- a/NSE1 Important Dates.xlsx
+++ b/NSE1 Important Dates.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="142">
   <si>
     <t>Country</t>
   </si>
@@ -440,12 +440,6 @@
   </si>
   <si>
     <t>Jamhuri Day</t>
-  </si>
-  <si>
-    <t>JSB BDAY</t>
-  </si>
-  <si>
-    <t>JSB Dad BDAY</t>
   </si>
   <si>
     <t>Description</t>
@@ -542,49 +536,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF16AA06"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF16AA06"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -911,7 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1796875" customWidth="1"/>
@@ -935,7 +887,7 @@
         <v>129</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -952,7 +904,7 @@
         <v>130</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1422,10 +1374,10 @@
         <v>5</v>
       </c>
       <c r="B36" s="5">
-        <v>46230</v>
+        <v>46371</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>132</v>
@@ -1433,30 +1385,30 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B37" s="5">
-        <v>46371</v>
+        <v>46073</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>139</v>
+        <v>85</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B38" s="5">
-        <v>46073</v>
+      <c r="B38" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>85</v>
+        <v>133</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1464,10 +1416,10 @@
         <v>6</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>133</v>
+        <v>86</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>132</v>
@@ -1478,10 +1430,10 @@
         <v>6</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>132</v>
@@ -1492,10 +1444,10 @@
         <v>6</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>134</v>
+        <v>87</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>132</v>
@@ -1503,16 +1455,16 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1520,10 +1472,10 @@
         <v>7</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>130</v>
@@ -1534,13 +1486,13 @@
         <v>7</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -1548,10 +1500,10 @@
         <v>7</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>132</v>
@@ -1559,13 +1511,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>132</v>
@@ -1576,10 +1528,10 @@
         <v>8</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>132</v>
@@ -1590,10 +1542,10 @@
         <v>8</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>132</v>
@@ -1604,10 +1556,10 @@
         <v>8</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>132</v>
@@ -1615,16 +1567,16 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
@@ -1632,27 +1584,27 @@
         <v>9</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
@@ -1660,10 +1612,10 @@
         <v>10</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>130</v>
@@ -1674,10 +1626,10 @@
         <v>10</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>130</v>
@@ -1688,13 +1640,13 @@
         <v>10</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -1702,13 +1654,13 @@
         <v>10</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
@@ -1716,10 +1668,10 @@
         <v>10</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>132</v>
@@ -1733,7 +1685,7 @@
         <v>20</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>132</v>
@@ -1744,10 +1696,10 @@
         <v>10</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>132</v>
@@ -1758,10 +1710,10 @@
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>132</v>
@@ -1769,16 +1721,16 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
@@ -1786,24 +1738,22 @@
         <v>11</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>130</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="D62" s="2"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D63" s="2"/>
     </row>
@@ -1812,10 +1762,10 @@
         <v>11</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D64" s="2"/>
     </row>
@@ -1824,10 +1774,10 @@
         <v>11</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D65" s="2"/>
     </row>
@@ -1836,10 +1786,10 @@
         <v>11</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D66" s="2"/>
     </row>
@@ -1851,19 +1801,21 @@
         <v>51</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D67" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>132</v>
@@ -1874,10 +1826,10 @@
         <v>11</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>132</v>
@@ -1888,10 +1840,10 @@
         <v>11</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>132</v>
@@ -1902,10 +1854,10 @@
         <v>11</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>132</v>
@@ -1916,10 +1868,10 @@
         <v>11</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>132</v>
@@ -1930,10 +1882,10 @@
         <v>11</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>132</v>
@@ -1941,13 +1893,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>132</v>
@@ -1955,13 +1907,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>132</v>
@@ -1972,10 +1924,10 @@
         <v>13</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>132</v>
@@ -1983,13 +1935,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>132</v>
@@ -2000,10 +1952,10 @@
         <v>14</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>132</v>
@@ -2017,7 +1969,7 @@
         <v>20</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>132</v>
@@ -2028,10 +1980,10 @@
         <v>14</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>132</v>
@@ -2042,10 +1994,10 @@
         <v>14</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>132</v>
@@ -2056,79 +2008,29 @@
         <v>14</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B84" s="5">
-        <v>46234</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D35 D37:D83 D85:D1048576 E1:E2">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
+  <conditionalFormatting sqref="D1:D1048576 E1:E2">
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
       <formula>"Postponed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="equal">
-      <formula>"Executed"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D36">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"Yet to Happen"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"Postponed"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
-      <formula>"Executed"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D84">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <formula>"Yet to Happen"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"Postponed"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
       <formula>"Executed"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D84">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D82">
       <formula1>"Executed, Postponed, Yet to Happen"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
new dates added - SA
</commit_message>
<xml_diff>
--- a/NSE1 Important Dates.xlsx
+++ b/NSE1 Important Dates.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="143">
   <si>
     <t>Country</t>
   </si>
@@ -223,12 +223,6 @@
     <t>Ronin &amp; Ntorq Launch</t>
   </si>
   <si>
-    <t>Ramadan Advertisements in TV and Social Media</t>
-  </si>
-  <si>
-    <t>Local Football sponsor with HLX range promotions</t>
-  </si>
-  <si>
     <t>XL 100  Dealer launch</t>
   </si>
   <si>
@@ -292,9 +286,6 @@
     <t>AOG 80kms ride to Mazagan Beach</t>
   </si>
   <si>
-    <t>Anniversary Celebration / Mass Delivery</t>
-  </si>
-  <si>
     <t>Apache AOG rides &amp; stunt show at Sindibad</t>
   </si>
   <si>
@@ -313,9 +304,6 @@
     <t>Virtual Distributor Conference</t>
   </si>
   <si>
-    <t>Virtual Distributor Conference 2.0</t>
-  </si>
-  <si>
     <t>TVS South Africa Country Launch</t>
   </si>
   <si>
@@ -328,21 +316,9 @@
     <t>Store Inaugration  Centurion, Pretoria,</t>
   </si>
   <si>
-    <t>Tie ups with Riding School</t>
-  </si>
-  <si>
-    <t>Store Inaugration  Ekrold, Durban</t>
-  </si>
-  <si>
     <t>HLX Day-Cape Town</t>
   </si>
   <si>
-    <t>India Visit- 7 Dealers</t>
-  </si>
-  <si>
-    <t>Store Inaugration  Tex,George</t>
-  </si>
-  <si>
     <t>HLX Day – Dar es Salaam</t>
   </si>
   <si>
@@ -439,20 +415,47 @@
     <t xml:space="preserve">Tris academy launch </t>
   </si>
   <si>
-    <t>Jamhuri Day</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
     <t xml:space="preserve">The event went rather well with over 200 people having to show what they are made of as mechanics. Winner gets an all expense paid trip to India </t>
+  </si>
+  <si>
+    <t>Q1 Townhall</t>
+  </si>
+  <si>
+    <t>Apache RTR 310 Launch</t>
+  </si>
+  <si>
+    <t>TVS Apache RTR 310 Morocco Launch marked TVS Motor Company’s entry into Africa’s premium motorcycle segment. The launch introduced the high-performance RTR 310 as a flagship “Track to Road” model for the growing 200–350cc market in Morocco.</t>
+  </si>
+  <si>
+    <t>The TVS King Deluxe Plus was introduced in Fort Dauphin, Madagascar, by late March 2026, highlighted as a strong and durable three-wheeler for the city's hilly terrain. This launch expands the presence of TVS Motor Company in Madagascar, featuring a reliable 3W designed for both passenger and commercial use throughout the island.</t>
+  </si>
+  <si>
+    <t>Bikers WareHouse Store Inauguration</t>
+  </si>
+  <si>
+    <t>I-Qube Launch</t>
+  </si>
+  <si>
+    <t>NTORQ150 &amp; RAIDER i-Go Launch</t>
+  </si>
+  <si>
+    <t>Riding School Collaboration with King Donut</t>
+  </si>
+  <si>
+    <t>Riding School Collaboration with Prestige Bikes</t>
+  </si>
+  <si>
+    <t>TVS Centurion 3S inaugartion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,6 +471,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -477,7 +487,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -511,11 +521,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -532,6 +557,8 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -863,14 +890,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1796875" customWidth="1"/>
     <col min="2" max="2" width="14.54296875" customWidth="1"/>
     <col min="3" max="3" width="66.453125" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" customWidth="1"/>
-    <col min="5" max="5" width="32.08984375" customWidth="1"/>
+    <col min="5" max="5" width="124.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -884,10 +911,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -901,10 +928,10 @@
         <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -918,7 +945,7 @@
         <v>56</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -932,7 +959,7 @@
         <v>57</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -946,7 +973,7 @@
         <v>58</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -960,7 +987,7 @@
         <v>59</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -974,7 +1001,7 @@
         <v>60</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -988,7 +1015,7 @@
         <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1002,7 +1029,7 @@
         <v>62</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1016,7 +1043,7 @@
         <v>63</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1030,7 +1057,7 @@
         <v>64</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1044,7 +1071,7 @@
         <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1058,7 +1085,7 @@
         <v>66</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1066,13 +1093,13 @@
         <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1080,13 +1107,13 @@
         <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1094,41 +1121,41 @@
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>30</v>
+        <v>5</v>
+      </c>
+      <c r="B18" s="3">
+        <v>46079</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1136,27 +1163,27 @@
         <v>5</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="3">
-        <v>46079</v>
+      <c r="B20" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1164,13 +1191,13 @@
         <v>5</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -1178,13 +1205,13 @@
         <v>5</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>138</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -1192,13 +1219,13 @@
         <v>5</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -1206,13 +1233,13 @@
         <v>5</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -1220,13 +1247,13 @@
         <v>5</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>74</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1234,13 +1261,13 @@
         <v>5</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1248,13 +1275,13 @@
         <v>5</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -1262,13 +1289,13 @@
         <v>5</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1276,13 +1303,13 @@
         <v>5</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1290,13 +1317,13 @@
         <v>5</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1304,13 +1331,13 @@
         <v>5</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1318,279 +1345,285 @@
         <v>5</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>81</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>30</v>
+        <v>6</v>
+      </c>
+      <c r="B34" s="5">
+        <v>46073</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B36" s="5">
-        <v>46371</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>139</v>
-      </c>
       <c r="D36" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B37" s="5">
-        <v>46073</v>
+      <c r="B37" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>133</v>
+        <v>85</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>88</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>91</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>92</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>93</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>24</v>
+        <v>9</v>
+      </c>
+      <c r="B48" s="5">
+        <v>46133</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
@@ -1598,125 +1631,125 @@
         <v>10</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>99</v>
+      <c r="B53" s="5">
+        <v>46136</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>140</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>100</v>
+      <c r="B54" s="5">
+        <v>46136</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>141</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>101</v>
+      <c r="B55" s="5">
+        <v>46137</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>142</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>19</v>
+      <c r="B56" s="5">
+        <v>46151</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>20</v>
+      <c r="B57" s="5">
+        <v>46188</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>104</v>
+      <c r="B58" s="5">
+        <v>46191</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>105</v>
+      <c r="B59" s="5">
+        <v>46193</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>139</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -1724,24 +1757,22 @@
         <v>11</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>130</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="D61" s="2"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D62" s="2"/>
     </row>
@@ -1750,10 +1781,10 @@
         <v>11</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D63" s="2"/>
     </row>
@@ -1762,10 +1793,10 @@
         <v>11</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D64" s="2"/>
     </row>
@@ -1774,10 +1805,10 @@
         <v>11</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D65" s="2"/>
     </row>
@@ -1789,22 +1820,24 @@
         <v>51</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D66" s="2"/>
+        <v>105</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -1812,13 +1845,13 @@
         <v>11</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -1826,13 +1859,13 @@
         <v>11</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -1840,13 +1873,13 @@
         <v>11</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -1854,13 +1887,13 @@
         <v>11</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -1868,41 +1901,41 @@
         <v>11</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
@@ -1910,27 +1943,27 @@
         <v>13</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
@@ -1938,13 +1971,13 @@
         <v>14</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
@@ -1955,10 +1988,10 @@
         <v>20</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
@@ -1966,13 +1999,13 @@
         <v>14</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
@@ -1980,13 +2013,13 @@
         <v>14</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
@@ -1994,31 +2027,17 @@
         <v>14</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D1048576 E1:E2">
+  <conditionalFormatting sqref="E1:E2 E35 D1:D1048576">
     <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
@@ -2030,7 +2049,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D82">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D81">
       <formula1>"Executed, Postponed, Yet to Happen"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
New dates for some cocuntries
</commit_message>
<xml_diff>
--- a/NSE1 Important Dates.xlsx
+++ b/NSE1 Important Dates.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$88</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="147">
   <si>
     <t>Country</t>
   </si>
@@ -399,12 +399,6 @@
     <t>Bikers WareHouse Store Inauguration</t>
   </si>
   <si>
-    <t>I-Qube Launch</t>
-  </si>
-  <si>
-    <t>NTORQ150 &amp; RAIDER i-Go Launch</t>
-  </si>
-  <si>
     <t>Riding School Collaboration with King Donut</t>
   </si>
   <si>
@@ -420,9 +414,6 @@
     <t>Zambia Product line Launch</t>
   </si>
   <si>
-    <t>HLX DAY</t>
-  </si>
-  <si>
     <t>Livingstone Riders Event</t>
   </si>
   <si>
@@ -442,6 +433,36 @@
   </si>
   <si>
     <t>RR 310 Launch &amp; AOG Flag off</t>
+  </si>
+  <si>
+    <t>HLX DAY Kisangani</t>
+  </si>
+  <si>
+    <t>EKROLD - Duran Dealer opening &amp; Activation</t>
+  </si>
+  <si>
+    <t>George Dealer Activation Program</t>
+  </si>
+  <si>
+    <t>Breakfast ride with Apache owners and Women Riders</t>
+  </si>
+  <si>
+    <t>Tamatave Coco Opening</t>
+  </si>
+  <si>
+    <t>Fort Dhaupin Festival Mandrae Participation</t>
+  </si>
+  <si>
+    <t>11-15-May-2026</t>
+  </si>
+  <si>
+    <t>Executed Successfully</t>
+  </si>
+  <si>
+    <t>TVS Centurion Inauguration &amp; Test Ride</t>
+  </si>
+  <si>
+    <t>Boda Girls Launch</t>
   </si>
 </sst>
 </file>
@@ -883,7 +904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1796875" customWidth="1"/>
@@ -1002,7 +1023,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>56</v>
@@ -1033,7 +1054,7 @@
         <v>46185</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>111</v>
@@ -1103,7 +1124,7 @@
         <v>46158</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>111</v>
@@ -1131,7 +1152,7 @@
         <v>46203</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>111</v>
@@ -1260,7 +1281,7 @@
         <v>67</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1268,10 +1289,10 @@
         <v>5</v>
       </c>
       <c r="B27" s="5">
-        <v>46188</v>
+        <v>46163</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>68</v>
+        <v>146</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>111</v>
@@ -1282,10 +1303,10 @@
         <v>5</v>
       </c>
       <c r="B28" s="5">
-        <v>46179</v>
+        <v>46188</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>139</v>
+        <v>68</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>111</v>
@@ -1296,10 +1317,10 @@
         <v>5</v>
       </c>
       <c r="B29" s="5">
-        <v>46201</v>
+        <v>46193</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>69</v>
+        <v>136</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>111</v>
@@ -1310,10 +1331,10 @@
         <v>5</v>
       </c>
       <c r="B30" s="5">
-        <v>46205</v>
+        <v>46201</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>111</v>
@@ -1324,10 +1345,10 @@
         <v>5</v>
       </c>
       <c r="B31" s="5">
-        <v>46399</v>
+        <v>46205</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>111</v>
@@ -1338,10 +1359,10 @@
         <v>5</v>
       </c>
       <c r="B32" s="5">
-        <v>46198</v>
+        <v>46399</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>111</v>
@@ -1349,33 +1370,30 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33" s="5">
-        <v>46073</v>
+        <v>46198</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>28</v>
+      <c r="B34" s="5">
+        <v>46073</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>112</v>
+        <v>73</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -1383,13 +1401,16 @@
         <v>6</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1397,13 +1418,13 @@
         <v>6</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1411,10 +1432,10 @@
         <v>6</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>111</v>
@@ -1422,58 +1443,55 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>31</v>
+        <v>6</v>
+      </c>
+      <c r="B38" s="5">
+        <v>46163</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>76</v>
+        <v>140</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>6</v>
+      </c>
+      <c r="B40" s="5">
+        <v>46192</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>42</v>
+        <v>6</v>
+      </c>
+      <c r="B41" s="5">
+        <v>46198</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>78</v>
+        <v>142</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>111</v>
@@ -1483,53 +1501,56 @@
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B42" s="5">
-        <v>46151</v>
+      <c r="B42" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>136</v>
+        <v>76</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B43" s="5">
-        <v>46165</v>
+      <c r="B43" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>135</v>
+        <v>77</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B44" s="5">
-        <v>46249</v>
+      <c r="B44" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>111</v>
@@ -1537,13 +1558,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
+      </c>
+      <c r="B46" s="5">
+        <v>46151</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>111</v>
@@ -1551,13 +1572,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>30</v>
+        <v>7</v>
+      </c>
+      <c r="B47" s="5">
+        <v>46165</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>111</v>
@@ -1565,257 +1586,260 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="5">
+        <v>46249</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B52" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="2" t="s">
+      <c r="D52" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B53" s="5">
         <v>46133</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="D53" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B54" s="5">
-        <v>46136</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>127</v>
+      <c r="B54" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B55" s="5">
-        <v>46136</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>128</v>
+      <c r="B55" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B56" s="5">
-        <v>46137</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>129</v>
+      <c r="B56" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B57" s="5">
-        <v>46151</v>
+      <c r="B57" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="5">
-        <v>46188</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>124</v>
+        <v>46136</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>125</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B59" s="5">
-        <v>46191</v>
+        <v>46136</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B60" s="5">
-        <v>46193</v>
+        <v>46137</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>46</v>
+        <v>10</v>
+      </c>
+      <c r="B61" s="5">
+        <v>46151</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
+      </c>
+      <c r="B62" s="5">
+        <v>46164</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="B63" s="5">
+        <v>46188</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>91</v>
+        <v>10</v>
+      </c>
+      <c r="B64" s="5">
+        <v>46180</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>92</v>
+        <v>10</v>
+      </c>
+      <c r="B65" s="5">
+        <v>46193</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>139</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -1823,13 +1847,13 @@
         <v>11</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -1837,13 +1861,13 @@
         <v>11</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -1851,10 +1875,10 @@
         <v>11</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>110</v>
@@ -1865,10 +1889,10 @@
         <v>11</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>110</v>
@@ -1879,10 +1903,10 @@
         <v>11</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>110</v>
@@ -1893,13 +1917,13 @@
         <v>11</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -1907,10 +1931,10 @@
         <v>11</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>111</v>
@@ -1921,52 +1945,52 @@
         <v>11</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>111</v>
@@ -1974,41 +1998,41 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B78" s="5">
-        <v>46132</v>
+        <v>11</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>131</v>
+        <v>100</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>111</v>
@@ -2016,13 +2040,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B80" s="5">
-        <v>46164</v>
+        <v>13</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>111</v>
@@ -2030,13 +2054,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B81" s="5">
-        <v>46218</v>
+        <v>13</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>111</v>
@@ -2046,33 +2070,103 @@
       <c r="A82" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="5">
-        <v>46183</v>
+      <c r="B82" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="5">
+        <v>46132</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B85" s="5">
+        <v>46164</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B86" s="5">
+        <v>46218</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B87" s="5">
+        <v>46183</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C88" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>111</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E83"/>
-  <conditionalFormatting sqref="E1:E2 E34 E48 D1:D1048576">
+  <autoFilter ref="A1:E88"/>
+  <conditionalFormatting sqref="E1:E2 E35 D1:D1048576 E52:E53">
     <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
@@ -2084,7 +2178,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D83">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D88">
       <formula1>"Executed, Postponed, Yet to Happen"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>